<commit_message>
Added database_number to resulting database and implemented it
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/Australia_Mataranka.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/Australia_Mataranka.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\Gesammelte_Datenbanken\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F3726BF-A480-4E47-A416-FB3E99D14C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{978F2D15-E204-4CC4-B7CB-9D2850E82216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{98FE92FD-BA3C-4C93-BCFC-8E434AAD9374}"/>
+    <workbookView xWindow="2160" yWindow="2160" windowWidth="21600" windowHeight="11295" xr2:uid="{98FE92FD-BA3C-4C93-BCFC-8E434AAD9374}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Completed Database for all databases as of now
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/Australia_Mataranka.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/Australia_Mataranka.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\Gesammelte_Datenbanken\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{978F2D15-E204-4CC4-B7CB-9D2850E82216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{738248BB-CF48-440A-B183-9DC23FFC93EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2160" yWindow="2160" windowWidth="21600" windowHeight="11295" xr2:uid="{98FE92FD-BA3C-4C93-BCFC-8E434AAD9374}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{98FE92FD-BA3C-4C93-BCFC-8E434AAD9374}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -197,12 +197,6 @@
     <t>RN034903</t>
   </si>
   <si>
-    <t>Bore/Spring</t>
-  </si>
-  <si>
-    <t>CLA flow path</t>
-  </si>
-  <si>
     <t>CLA Formation</t>
   </si>
   <si>
@@ -228,24 +222,6 @@
   </si>
   <si>
     <t>Source</t>
-  </si>
-  <si>
-    <t>Ca (mg/L)</t>
-  </si>
-  <si>
-    <t>Mg (mg/L)</t>
-  </si>
-  <si>
-    <t>K (mg/L)</t>
-  </si>
-  <si>
-    <t>Na (mg/L)</t>
-  </si>
-  <si>
-    <t>Cl (mg/L)</t>
-  </si>
-  <si>
-    <t>SO4 (mg/L)</t>
   </si>
   <si>
     <r>
@@ -442,10 +418,34 @@
     </r>
   </si>
   <si>
-    <t>Alkalinity (meq/L)</t>
-  </si>
-  <si>
     <t>Database_number</t>
+  </si>
+  <si>
+    <t>CLA_flow_path</t>
+  </si>
+  <si>
+    <t>Bore_Spring</t>
+  </si>
+  <si>
+    <t>K_mg-L</t>
+  </si>
+  <si>
+    <t>Mg_mg-L</t>
+  </si>
+  <si>
+    <t>Ca_mg-L</t>
+  </si>
+  <si>
+    <t>Na_mg-L</t>
+  </si>
+  <si>
+    <t>Cl_mg-L</t>
+  </si>
+  <si>
+    <t>SO4_mg-L</t>
+  </si>
+  <si>
+    <t>Alkalinity_meq-L</t>
   </si>
 </sst>
 </file>
@@ -936,55 +936,55 @@
   <sheetData>
     <row r="1" spans="1:17" ht="16.5">
       <c r="A1" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="D1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="D1" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>58</v>
-      </c>
       <c r="G1" s="8" t="s">
-        <v>65</v>
+        <v>107</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>66</v>
+        <v>106</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>68</v>
+        <v>108</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>69</v>
+        <v>109</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="N1" s="9" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="O1" s="9" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="Q1" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:17">
@@ -992,7 +992,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C2" t="s">
         <v>1</v>
@@ -1034,7 +1034,7 @@
         <v>-44.1</v>
       </c>
       <c r="P2" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q2">
         <v>9</v>
@@ -1045,7 +1045,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
@@ -1087,7 +1087,7 @@
         <v>-53.4</v>
       </c>
       <c r="P3" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q3">
         <v>9</v>
@@ -1098,7 +1098,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C4" t="s">
         <v>1</v>
@@ -1140,7 +1140,7 @@
         <v>-54.5</v>
       </c>
       <c r="P4" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q4">
         <v>9</v>
@@ -1151,7 +1151,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C5" t="s">
         <v>1</v>
@@ -1166,7 +1166,7 @@
         <v>-14.710452999999999</v>
       </c>
       <c r="G5" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="H5">
         <v>31.2</v>
@@ -1193,7 +1193,7 @@
         <v>-52.3</v>
       </c>
       <c r="P5" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q5">
         <v>9</v>
@@ -1204,7 +1204,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C6" t="s">
         <v>1</v>
@@ -1246,7 +1246,7 @@
         <v>-54.8</v>
       </c>
       <c r="P6" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q6">
         <v>9</v>
@@ -1257,7 +1257,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C7" t="s">
         <v>1</v>
@@ -1299,7 +1299,7 @@
         <v>-47.1</v>
       </c>
       <c r="P7" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q7">
         <v>9</v>
@@ -1310,7 +1310,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C8" t="s">
         <v>1</v>
@@ -1331,7 +1331,7 @@
         <v>30</v>
       </c>
       <c r="I8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J8">
         <v>4</v>
@@ -1352,7 +1352,7 @@
         <v>-42.3</v>
       </c>
       <c r="P8" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q8">
         <v>9</v>
@@ -1363,7 +1363,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C9" t="s">
         <v>1</v>
@@ -1405,7 +1405,7 @@
         <v>-54.7</v>
       </c>
       <c r="P9" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q9">
         <v>9</v>
@@ -1416,7 +1416,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
         <v>1</v>
@@ -1458,7 +1458,7 @@
         <v>-46.7</v>
       </c>
       <c r="P10" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q10">
         <v>9</v>
@@ -1469,7 +1469,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C11" t="s">
         <v>1</v>
@@ -1484,7 +1484,7 @@
         <v>-14.411049999999999</v>
       </c>
       <c r="G11" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="H11">
         <v>24.5</v>
@@ -1511,7 +1511,7 @@
         <v>-51.6</v>
       </c>
       <c r="P11" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q11">
         <v>9</v>
@@ -1522,7 +1522,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C12" t="s">
         <v>1</v>
@@ -1564,7 +1564,7 @@
         <v>-54.7</v>
       </c>
       <c r="P12" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q12">
         <v>9</v>
@@ -1575,7 +1575,7 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C13" t="s">
         <v>1</v>
@@ -1590,7 +1590,7 @@
         <v>-14.503927790000001</v>
       </c>
       <c r="G13" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="H13">
         <v>39.299999999999997</v>
@@ -1617,7 +1617,7 @@
         <v>-51.14</v>
       </c>
       <c r="P13" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q13">
         <v>9</v>
@@ -1628,7 +1628,7 @@
         <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C14" t="s">
         <v>1</v>
@@ -1670,7 +1670,7 @@
         <v>-50.2</v>
       </c>
       <c r="P14" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q14">
         <v>9</v>
@@ -1681,7 +1681,7 @@
         <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C15" t="s">
         <v>1</v>
@@ -1723,7 +1723,7 @@
         <v>-46.7</v>
       </c>
       <c r="P15" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q15">
         <v>9</v>
@@ -1734,7 +1734,7 @@
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C16" t="s">
         <v>1</v>
@@ -1776,7 +1776,7 @@
         <v>-49.4</v>
       </c>
       <c r="P16" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q16">
         <v>9</v>
@@ -1787,7 +1787,7 @@
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C17" t="s">
         <v>1</v>
@@ -1817,7 +1817,7 @@
         <v>4.5</v>
       </c>
       <c r="L17" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M17">
         <v>7.4</v>
@@ -1829,7 +1829,7 @@
         <v>-50.81</v>
       </c>
       <c r="P17" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q17">
         <v>9</v>
@@ -1840,7 +1840,7 @@
         <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C18" t="s">
         <v>1</v>
@@ -1882,7 +1882,7 @@
         <v>-45.7</v>
       </c>
       <c r="P18" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q18">
         <v>9</v>
@@ -1893,7 +1893,7 @@
         <v>16</v>
       </c>
       <c r="B19" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C19" t="s">
         <v>1</v>
@@ -1923,7 +1923,7 @@
         <v>8.6</v>
       </c>
       <c r="L19" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M19">
         <v>6.7</v>
@@ -1935,7 +1935,7 @@
         <v>-52.55</v>
       </c>
       <c r="P19" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q19">
         <v>9</v>
@@ -1946,7 +1946,7 @@
         <v>17</v>
       </c>
       <c r="B20" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C20" t="s">
         <v>1</v>
@@ -1976,7 +1976,7 @@
         <v>6.1</v>
       </c>
       <c r="L20" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M20">
         <v>7.4</v>
@@ -1988,7 +1988,7 @@
         <v>-51.67</v>
       </c>
       <c r="P20" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q20">
         <v>9</v>
@@ -1999,7 +1999,7 @@
         <v>18</v>
       </c>
       <c r="B21" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C21" t="s">
         <v>1</v>
@@ -2029,7 +2029,7 @@
         <v>5.6</v>
       </c>
       <c r="L21" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M21">
         <v>9.6</v>
@@ -2041,7 +2041,7 @@
         <v>-49.96</v>
       </c>
       <c r="P21" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q21">
         <v>9</v>
@@ -2052,7 +2052,7 @@
         <v>19</v>
       </c>
       <c r="B22" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C22" t="s">
         <v>1</v>
@@ -2082,7 +2082,7 @@
         <v>5.4</v>
       </c>
       <c r="L22" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M22">
         <v>7.6</v>
@@ -2094,7 +2094,7 @@
         <v>-49.47</v>
       </c>
       <c r="P22" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q22">
         <v>9</v>
@@ -2105,7 +2105,7 @@
         <v>20</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C23" t="s">
         <v>1</v>
@@ -2147,7 +2147,7 @@
         <v>-48.8</v>
       </c>
       <c r="P23" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q23">
         <v>9</v>
@@ -2158,7 +2158,7 @@
         <v>21</v>
       </c>
       <c r="B24" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C24" t="s">
         <v>1</v>
@@ -2200,7 +2200,7 @@
         <v>-40.700000000000003</v>
       </c>
       <c r="P24" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q24">
         <v>9</v>
@@ -2211,7 +2211,7 @@
         <v>22</v>
       </c>
       <c r="B25" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C25" t="s">
         <v>1</v>
@@ -2253,7 +2253,7 @@
         <v>-51.3</v>
       </c>
       <c r="P25" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q25">
         <v>9</v>
@@ -2264,7 +2264,7 @@
         <v>23</v>
       </c>
       <c r="B26" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C26" t="s">
         <v>1</v>
@@ -2306,7 +2306,7 @@
         <v>-47.4</v>
       </c>
       <c r="P26" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q26">
         <v>9</v>
@@ -2317,7 +2317,7 @@
         <v>24</v>
       </c>
       <c r="B27" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C27" t="s">
         <v>1</v>
@@ -2359,7 +2359,7 @@
         <v>-51.1</v>
       </c>
       <c r="P27" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q27">
         <v>9</v>
@@ -2370,7 +2370,7 @@
         <v>25</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C28" t="s">
         <v>1</v>
@@ -2412,7 +2412,7 @@
         <v>-48.1</v>
       </c>
       <c r="P28" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q28">
         <v>9</v>
@@ -2423,7 +2423,7 @@
         <v>26</v>
       </c>
       <c r="B29" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C29" t="s">
         <v>1</v>
@@ -2465,7 +2465,7 @@
         <v>-53.2</v>
       </c>
       <c r="P29" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q29">
         <v>9</v>
@@ -2476,7 +2476,7 @@
         <v>27</v>
       </c>
       <c r="B30" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C30" t="s">
         <v>1</v>
@@ -2518,7 +2518,7 @@
         <v>-51.29</v>
       </c>
       <c r="P30" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q30">
         <v>9</v>
@@ -2529,7 +2529,7 @@
         <v>28</v>
       </c>
       <c r="B31" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C31" t="s">
         <v>1</v>
@@ -2571,7 +2571,7 @@
         <v>-53.8</v>
       </c>
       <c r="P31" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q31">
         <v>9</v>
@@ -2582,7 +2582,7 @@
         <v>29</v>
       </c>
       <c r="B32" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C32" t="s">
         <v>1</v>
@@ -2624,7 +2624,7 @@
         <v>-48.4</v>
       </c>
       <c r="P32" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q32">
         <v>9</v>
@@ -2635,7 +2635,7 @@
         <v>30</v>
       </c>
       <c r="B33" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C33" t="s">
         <v>1</v>
@@ -2677,7 +2677,7 @@
         <v>-49.69</v>
       </c>
       <c r="P33" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q33">
         <v>9</v>
@@ -2688,7 +2688,7 @@
         <v>31</v>
       </c>
       <c r="B34" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C34" t="s">
         <v>1</v>
@@ -2730,7 +2730,7 @@
         <v>-56.3</v>
       </c>
       <c r="P34" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q34">
         <v>9</v>
@@ -2741,7 +2741,7 @@
         <v>31</v>
       </c>
       <c r="B35" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C35" t="s">
         <v>1</v>
@@ -2771,7 +2771,7 @@
         <v>3.8</v>
       </c>
       <c r="L35" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M35">
         <v>6.6</v>
@@ -2783,7 +2783,7 @@
         <v>-56.1</v>
       </c>
       <c r="P35" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q35">
         <v>9</v>
@@ -2794,7 +2794,7 @@
         <v>32</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>1</v>
@@ -2824,7 +2824,7 @@
         <v>8</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M36" s="2">
         <v>7</v>
@@ -2836,7 +2836,7 @@
         <v>-50.38</v>
       </c>
       <c r="P36" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q36">
         <v>9</v>
@@ -2847,7 +2847,7 @@
         <v>33</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>1</v>
@@ -2862,22 +2862,22 @@
         <v>-14.45491</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="M37" s="6"/>
       <c r="N37" s="6">
@@ -2887,7 +2887,7 @@
         <v>-45</v>
       </c>
       <c r="P37" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q37">
         <v>9</v>
@@ -2898,7 +2898,7 @@
         <v>34</v>
       </c>
       <c r="B38" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C38" t="s">
         <v>1</v>
@@ -2928,7 +2928,7 @@
         <v>12.9</v>
       </c>
       <c r="L38" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M38">
         <v>7</v>
@@ -2940,7 +2940,7 @@
         <v>-48.68</v>
       </c>
       <c r="P38" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q38">
         <v>9</v>
@@ -2951,7 +2951,7 @@
         <v>35</v>
       </c>
       <c r="B39" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C39" t="s">
         <v>1</v>
@@ -2993,7 +2993,7 @@
         <v>-49.1</v>
       </c>
       <c r="P39" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q39">
         <v>9</v>
@@ -3004,7 +3004,7 @@
         <v>36</v>
       </c>
       <c r="B40" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C40" t="s">
         <v>1</v>
@@ -3034,7 +3034,7 @@
         <v>6.3</v>
       </c>
       <c r="L40" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M40">
         <v>7.6</v>
@@ -3046,7 +3046,7 @@
         <v>-48.37</v>
       </c>
       <c r="P40" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q40">
         <v>9</v>
@@ -3057,7 +3057,7 @@
         <v>37</v>
       </c>
       <c r="B41" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C41" t="s">
         <v>38</v>
@@ -3099,7 +3099,7 @@
         <v>-51.4</v>
       </c>
       <c r="P41" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q41">
         <v>9</v>
@@ -3110,7 +3110,7 @@
         <v>39</v>
       </c>
       <c r="B42" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C42" t="s">
         <v>38</v>
@@ -3152,7 +3152,7 @@
         <v>-52.4</v>
       </c>
       <c r="P42" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q42">
         <v>9</v>
@@ -3163,7 +3163,7 @@
         <v>40</v>
       </c>
       <c r="B43" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C43" t="s">
         <v>1</v>
@@ -3205,7 +3205,7 @@
         <v>-47.1</v>
       </c>
       <c r="P43" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q43">
         <v>9</v>
@@ -3216,7 +3216,7 @@
         <v>41</v>
       </c>
       <c r="B44" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C44" t="s">
         <v>1</v>
@@ -3246,7 +3246,7 @@
         <v>5.3</v>
       </c>
       <c r="L44" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M44">
         <v>7.3</v>
@@ -3258,7 +3258,7 @@
         <v>-50.61</v>
       </c>
       <c r="P44" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q44">
         <v>9</v>
@@ -3269,7 +3269,7 @@
         <v>42</v>
       </c>
       <c r="B45" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C45" t="s">
         <v>1</v>
@@ -3311,7 +3311,7 @@
         <v>-46.7</v>
       </c>
       <c r="P45" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q45">
         <v>9</v>
@@ -3322,7 +3322,7 @@
         <v>43</v>
       </c>
       <c r="B46" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C46" t="s">
         <v>1</v>
@@ -3352,7 +3352,7 @@
         <v>4</v>
       </c>
       <c r="L46" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M46">
         <v>9.1</v>
@@ -3364,7 +3364,7 @@
         <v>-48.68</v>
       </c>
       <c r="P46" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q46">
         <v>9</v>
@@ -3375,7 +3375,7 @@
         <v>44</v>
       </c>
       <c r="B47" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C47" t="s">
         <v>1</v>
@@ -3405,7 +3405,7 @@
         <v>12.3</v>
       </c>
       <c r="L47" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M47">
         <v>8</v>
@@ -3417,7 +3417,7 @@
         <v>-52.75</v>
       </c>
       <c r="P47" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q47">
         <v>9</v>
@@ -3428,7 +3428,7 @@
         <v>45</v>
       </c>
       <c r="B48" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C48" t="s">
         <v>1</v>
@@ -3458,7 +3458,7 @@
         <v>19.5</v>
       </c>
       <c r="L48" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M48">
         <v>7.2</v>
@@ -3470,7 +3470,7 @@
         <v>-53.43</v>
       </c>
       <c r="P48" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q48">
         <v>9</v>
@@ -3481,7 +3481,7 @@
         <v>46</v>
       </c>
       <c r="B49" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C49" t="s">
         <v>1</v>
@@ -3511,7 +3511,7 @@
         <v>7.5</v>
       </c>
       <c r="L49" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M49">
         <v>8.1999999999999993</v>
@@ -3523,7 +3523,7 @@
         <v>-48.98</v>
       </c>
       <c r="P49" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q49">
         <v>9</v>
@@ -3534,7 +3534,7 @@
         <v>47</v>
       </c>
       <c r="B50" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C50" t="s">
         <v>1</v>
@@ -3576,7 +3576,7 @@
         <v>-50.1</v>
       </c>
       <c r="P50" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q50">
         <v>9</v>
@@ -3587,7 +3587,7 @@
         <v>48</v>
       </c>
       <c r="B51" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C51" t="s">
         <v>38</v>
@@ -3629,7 +3629,7 @@
         <v>-50.949999999999996</v>
       </c>
       <c r="P51" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q51">
         <v>9</v>
@@ -3640,7 +3640,7 @@
         <v>49</v>
       </c>
       <c r="B52" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C52" t="s">
         <v>1</v>
@@ -3670,7 +3670,7 @@
         <v>13.6</v>
       </c>
       <c r="L52" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M52">
         <v>6.8</v>
@@ -3682,7 +3682,7 @@
         <v>-47.41</v>
       </c>
       <c r="P52" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q52">
         <v>9</v>
@@ -3693,7 +3693,7 @@
         <v>50</v>
       </c>
       <c r="B53" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C53" t="s">
         <v>1</v>
@@ -3723,7 +3723,7 @@
         <v>6.3</v>
       </c>
       <c r="L53" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M53">
         <v>6.8</v>
@@ -3735,7 +3735,7 @@
         <v>-53.57</v>
       </c>
       <c r="P53" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q53">
         <v>9</v>
@@ -3746,7 +3746,7 @@
         <v>51</v>
       </c>
       <c r="B54" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C54" t="s">
         <v>1</v>
@@ -3776,7 +3776,7 @@
         <v>5.8</v>
       </c>
       <c r="L54" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M54">
         <v>7.4</v>
@@ -3788,7 +3788,7 @@
         <v>-48.34</v>
       </c>
       <c r="P54" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q54">
         <v>9</v>
@@ -3799,7 +3799,7 @@
         <v>52</v>
       </c>
       <c r="B55" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C55" t="s">
         <v>38</v>
@@ -3841,7 +3841,7 @@
         <v>-47.9</v>
       </c>
       <c r="P55" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q55">
         <v>9</v>
@@ -3849,10 +3849,10 @@
     </row>
     <row r="56" spans="1:17">
       <c r="A56" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B56" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C56" t="s">
         <v>1</v>
@@ -3882,7 +3882,7 @@
         <v>16.399999999999999</v>
       </c>
       <c r="L56" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="M56">
         <v>5.4</v>
@@ -3894,7 +3894,7 @@
         <v>-49.66</v>
       </c>
       <c r="P56" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q56">
         <v>9</v>
@@ -3905,7 +3905,7 @@
         <v>53</v>
       </c>
       <c r="B57" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C57" t="s">
         <v>1</v>
@@ -3947,7 +3947,7 @@
         <v>-52.07</v>
       </c>
       <c r="P57" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Q57">
         <v>9</v>
@@ -3955,13 +3955,13 @@
     </row>
     <row r="58" spans="1:17">
       <c r="A58" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B58" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C58" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="D58" s="1">
         <v>43392</v>
@@ -4000,7 +4000,7 @@
         <v>-8.69</v>
       </c>
       <c r="P58" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q58">
         <v>9</v>
@@ -4008,13 +4008,13 @@
     </row>
     <row r="59" spans="1:17">
       <c r="A59" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B59" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C59" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D59" s="1">
         <v>43397</v>
@@ -4053,7 +4053,7 @@
         <v>-8.41</v>
       </c>
       <c r="P59" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q59">
         <v>9</v>
@@ -4061,13 +4061,13 @@
     </row>
     <row r="60" spans="1:17">
       <c r="A60" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="B60" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C60" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D60" s="1">
         <v>43397</v>
@@ -4106,7 +4106,7 @@
         <v>-8.4</v>
       </c>
       <c r="P60" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q60">
         <v>9</v>
@@ -4114,13 +4114,13 @@
     </row>
     <row r="61" spans="1:17">
       <c r="A61" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="B61" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C61" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D61" s="1">
         <v>43397</v>
@@ -4159,7 +4159,7 @@
         <v>-7.92</v>
       </c>
       <c r="P61" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q61">
         <v>9</v>
@@ -4167,13 +4167,13 @@
     </row>
     <row r="62" spans="1:17">
       <c r="A62" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B62" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C62" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D62" s="1">
         <v>43397</v>
@@ -4212,7 +4212,7 @@
         <v>-8.3699999999999992</v>
       </c>
       <c r="P62" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q62">
         <v>9</v>
@@ -4220,13 +4220,13 @@
     </row>
     <row r="63" spans="1:17">
       <c r="A63" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="B63" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C63" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D63" s="1">
         <v>43398</v>
@@ -4265,7 +4265,7 @@
         <v>-8.4600000000000009</v>
       </c>
       <c r="P63" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q63">
         <v>9</v>
@@ -4273,13 +4273,13 @@
     </row>
     <row r="64" spans="1:17">
       <c r="A64" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B64" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C64" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D64" s="1">
         <v>43398</v>
@@ -4318,7 +4318,7 @@
         <v>-8.14</v>
       </c>
       <c r="P64" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q64">
         <v>9</v>
@@ -4326,13 +4326,13 @@
     </row>
     <row r="65" spans="1:17">
       <c r="A65" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="B65" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C65" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D65" s="1">
         <v>43399</v>
@@ -4371,7 +4371,7 @@
         <v>-8.3699999999999992</v>
       </c>
       <c r="P65" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q65">
         <v>9</v>
@@ -4379,13 +4379,13 @@
     </row>
     <row r="66" spans="1:17">
       <c r="A66" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B66" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C66" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D66" s="1">
         <v>43399</v>
@@ -4424,7 +4424,7 @@
         <v>-8.39</v>
       </c>
       <c r="P66" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q66">
         <v>9</v>
@@ -4432,13 +4432,13 @@
     </row>
     <row r="67" spans="1:17">
       <c r="A67" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="B67" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C67" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D67" s="1">
         <v>43403</v>
@@ -4477,7 +4477,7 @@
         <v>-8.44</v>
       </c>
       <c r="P67" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q67">
         <v>9</v>
@@ -4485,13 +4485,13 @@
     </row>
     <row r="68" spans="1:17">
       <c r="A68" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="B68" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C68" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D68" s="1">
         <v>43403</v>
@@ -4530,7 +4530,7 @@
         <v>-8.4499999999999993</v>
       </c>
       <c r="P68" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q68">
         <v>9</v>
@@ -4538,13 +4538,13 @@
     </row>
     <row r="69" spans="1:17">
       <c r="A69" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="B69" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C69" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D69" s="1">
         <v>43405</v>
@@ -4583,7 +4583,7 @@
         <v>-7</v>
       </c>
       <c r="P69" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q69">
         <v>9</v>
@@ -4591,13 +4591,13 @@
     </row>
     <row r="70" spans="1:17">
       <c r="A70" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="B70" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C70" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D70" s="1">
         <v>43405</v>
@@ -4636,7 +4636,7 @@
         <v>-8.5</v>
       </c>
       <c r="P70" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q70">
         <v>9</v>
@@ -4644,13 +4644,13 @@
     </row>
     <row r="71" spans="1:17">
       <c r="A71" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B71" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C71" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="D71" s="1">
         <v>43405</v>
@@ -4689,7 +4689,7 @@
         <v>-7.53</v>
       </c>
       <c r="P71" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q71">
         <v>9</v>
@@ -4697,13 +4697,13 @@
     </row>
     <row r="72" spans="1:17">
       <c r="A72" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="B72" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C72" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="D72" s="1">
         <v>43406</v>
@@ -4742,7 +4742,7 @@
         <v>-7.22</v>
       </c>
       <c r="P72" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q72">
         <v>9</v>
@@ -4750,13 +4750,13 @@
     </row>
     <row r="73" spans="1:17">
       <c r="A73" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="B73" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C73" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="D73" s="1">
         <v>43406</v>
@@ -4795,7 +4795,7 @@
         <v>-6.28</v>
       </c>
       <c r="P73" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q73">
         <v>9</v>
@@ -4803,13 +4803,13 @@
     </row>
     <row r="74" spans="1:17">
       <c r="A74" t="s">
+        <v>80</v>
+      </c>
+      <c r="B74" t="s">
         <v>88</v>
       </c>
-      <c r="B74" t="s">
-        <v>96</v>
-      </c>
       <c r="C74" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D74" s="1">
         <v>43407</v>
@@ -4848,7 +4848,7 @@
         <v>-7.53</v>
       </c>
       <c r="P74" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="Q74">
         <v>9</v>
@@ -4856,13 +4856,13 @@
     </row>
     <row r="75" spans="1:17">
       <c r="A75" t="s">
+        <v>81</v>
+      </c>
+      <c r="B75" t="s">
+        <v>88</v>
+      </c>
+      <c r="C75" t="s">
         <v>89</v>
-      </c>
-      <c r="B75" t="s">
-        <v>96</v>
-      </c>
-      <c r="C75" t="s">
-        <v>97</v>
       </c>
       <c r="D75" s="1">
         <v>43018</v>
@@ -4901,7 +4901,7 @@
         <v>-7.79</v>
       </c>
       <c r="P75" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="Q75">
         <v>9</v>
@@ -4909,13 +4909,13 @@
     </row>
     <row r="76" spans="1:17">
       <c r="A76" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="B76" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C76" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="D76" s="1">
         <v>43018</v>
@@ -4954,7 +4954,7 @@
         <v>-8.18</v>
       </c>
       <c r="P76" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="Q76">
         <v>9</v>
@@ -4962,13 +4962,13 @@
     </row>
     <row r="77" spans="1:17">
       <c r="A77" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="B77" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C77" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="D77" s="1">
         <v>43018</v>
@@ -5007,7 +5007,7 @@
         <v>-8.51</v>
       </c>
       <c r="P77" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="Q77">
         <v>9</v>
@@ -5015,13 +5015,13 @@
     </row>
     <row r="78" spans="1:17">
       <c r="A78" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B78" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C78" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="D78" s="1">
         <v>43018</v>
@@ -5060,7 +5060,7 @@
         <v>-7.94</v>
       </c>
       <c r="P78" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="Q78">
         <v>9</v>
@@ -5068,13 +5068,13 @@
     </row>
     <row r="79" spans="1:17">
       <c r="A79" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="B79" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C79" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D79" s="1">
         <v>43019</v>
@@ -5113,7 +5113,7 @@
         <v>-8.1999999999999993</v>
       </c>
       <c r="P79" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="Q79">
         <v>9</v>
@@ -5121,13 +5121,13 @@
     </row>
     <row r="80" spans="1:17">
       <c r="A80" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B80" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C80" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="D80" s="1">
         <v>43019</v>
@@ -5166,7 +5166,7 @@
         <v>-7.85</v>
       </c>
       <c r="P80" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="Q80">
         <v>9</v>
@@ -5174,13 +5174,13 @@
     </row>
     <row r="81" spans="1:17">
       <c r="A81" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B81" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C81" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D81" s="1">
         <v>43020</v>
@@ -5219,7 +5219,7 @@
         <v>-8.25</v>
       </c>
       <c r="P81" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="Q81">
         <v>9</v>
@@ -5227,13 +5227,13 @@
     </row>
     <row r="82" spans="1:17">
       <c r="A82" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="B82" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C82" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D82" s="1">
         <v>43020</v>
@@ -5272,7 +5272,7 @@
         <v>-8.31</v>
       </c>
       <c r="P82" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="Q82">
         <v>9</v>
@@ -5280,7 +5280,7 @@
     </row>
     <row r="83" spans="1:17">
       <c r="A83" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D83" s="1">
         <v>37742</v>
@@ -5313,13 +5313,13 @@
         <v>17</v>
       </c>
       <c r="N83" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="O83" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="P83" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="Q83">
         <v>9</v>
@@ -5327,7 +5327,7 @@
     </row>
     <row r="84" spans="1:17">
       <c r="A84" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D84" s="1">
         <v>37918</v>
@@ -5360,13 +5360,13 @@
         <v>16</v>
       </c>
       <c r="N84" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="O84" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="P84" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="Q84">
         <v>9</v>
@@ -5374,7 +5374,7 @@
     </row>
     <row r="85" spans="1:17">
       <c r="A85" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D85" s="1">
         <v>38217</v>
@@ -5407,13 +5407,13 @@
         <v>18</v>
       </c>
       <c r="N85" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="O85" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="P85" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="Q85">
         <v>9</v>

</xml_diff>